<commit_message>
fix(docs): fix UTF-8 encoding for Vietnamese characters in Rubric.xlsx
</commit_message>
<xml_diff>
--- a/Rubric.xlsx
+++ b/Rubric.xlsx
@@ -548,42 +548,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="85" customWidth="1" min="7" max="7"/>
+    <col width="90" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TR??NG ??I H?C T?N ??C TH?NG - KHOA C?NG NGH? TH?NG TIN</t>
+          <t>TRƯỜNG ĐẠI HỌC TÔN ĐỨC THẮNG - KHOA CÔNG NGHỆ THÔNG TIN</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>503073 ? L?P TR?NH WEB V? ?NG D?NG | FINAL PROJECT ? RUBRIC SELF-ASSESSMENT FORM</t>
+          <t>503073 – LẬP TRÌNH WEB VÀ ỨNG DỤNG | FINAL PROJECT – RUBRIC SELF-ASSESSMENT FORM</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>T?n ?? t?i:</t>
+          <t>Tên đề tài:</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>?ng d?ng Qu?n l? Ghi ch? Tr?c tuy?n (NoteApp)</t>
+          <t>Ứng dụng Quản lý Ghi chú Trực tuyến (NoteApp)</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>URL D? ?n:</t>
+          <t>URL Dự án:</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -595,29 +595,29 @@
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Th?nh vi?n 1:</t>
+          <t>Thành viên 1:</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>L? Ho?ng Tr? - MSSV: 524H0199 (trihoangle17)</t>
+          <t>Lê Hoàng Trí - MSSV: 524H0199 (trihoangle17)</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>T?i kho?n test ch?nh:</t>
+          <t>Tài khoản test chính:</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>demo@noteapp.local / Demo@123 (M?t kh?u ghi ch? kh?a: 1234)</t>
+          <t>demo@noteapp.local / Demo@123 (Mật khẩu ghi chú khóa: 1234)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Th?nh vi?n 2:</t>
+          <t>Thành viên 2:</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -627,7 +627,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>T?i kho?n test c?ng t?c:</t>
+          <t>Tài khoản test cộng tác:</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -649,7 +649,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>T?i kho?n test ch?a k?ch ho?t:</t>
+          <t>Tài khoản test chưa kích hoạt:</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -666,32 +666,32 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Nh?m Ch?c N?ng</t>
+          <t>Nhóm Chức Năng</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Ti?u Ch? ??nh Gi? (Criteria)</t>
+          <t>Tiêu Chí Đánh Giá (Criteria)</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>?i?m T?i ?a</t>
+          <t>Điểm Tối Đa</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>M?c ??t ???c</t>
+          <t>Mức Đạt Được</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>?i?m T? Ch?m</t>
+          <t>Điểm Tự Chấm</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Ghi Ch? Ki?m Th? &amp; Minh Ch?ng M? Ngu?n</t>
+          <t>Ghi Chú Kiểm Thử &amp; Minh Chứng Mã Nguồn</t>
         </is>
       </c>
     </row>
@@ -722,7 +722,7 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Email, display name, password (x2), Bcrypt hashing, auto-login, g?i token k?ch ho?t (AuthController.php:register)</t>
+          <t>Email, display name, password (x2), Bcrypt hashing, auto-login, gửi token kích hoạt (AuthController.php:register)</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>Banner c?nh b?o ch?a k?ch ho?t, k?ch ho?t qua link /activate?token=..., k?ch ho?t xong banner bi?n m?t</t>
+          <t>Banner cảnh báo chưa kích hoạt, kích hoạt qua link /activate?token=..., kích hoạt xong banner biến mất</t>
         </is>
       </c>
     </row>
@@ -784,7 +784,7 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Ch?a ??ng nh?p chuy?n v? /login, ??ng nh?p th?nh c?ng v?o homepage ghi ch?, ??ng xu?t an to?n</t>
+          <t>Chưa đăng nhập chuyển về /login, đăng nhập thành công vào homepage ghi chú, đăng xuất an toàn</t>
         </is>
       </c>
     </row>
@@ -815,7 +815,7 @@
       </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
-          <t>Kh?i ph?c qua link email ho?c m? OTP, ??t l?i m?t kh?u xong y?u c?u ??ng nh?p l?i</t>
+          <t>Khôi phục qua link email hoặc mã OTP, đặt lại mật khẩu xong yêu cầu đăng nhập lại</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>Xem display name, email v? avatar. Hi?n th? avatar m?c ??nh SVG khi ch?a upload</t>
+          <t>Xem display name, email và avatar. Hiển thị avatar mặc định SVG khi chưa upload</t>
         </is>
       </c>
     </row>
@@ -877,7 +877,7 @@
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>C?p nh?t display name, upload avatar c? ki?m tra MIME finfo, gi?i h?n 2MB, ??i t?n file ng?u nhi?n</t>
+          <t>Cập nhật display name, upload avatar có kiểm tra MIME finfo, giới hạn 2MB, đổi tên file ngẫu nhiên</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Nh?p m?t kh?u c? + m?t kh?u m?i (x2), t?i t?o session ID b?o m?t sau khi ??i</t>
+          <t>Nhập mật khẩu cũ + mật khẩu mới (x2), tái tạo session ID bảo mật sau khi đổi</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="G17" s="12" t="inlineStr">
         <is>
-          <t>T?y ch?nh c? ch? (small/medium/large), b?ng ch?n m?u n?n ghi ch?, chuy?n Light / Dark theme t?c th?</t>
+          <t>Tùy chỉnh cỡ chữ (small/medium/large), bảng chọn màu nền ghi chú, chuyển Light / Dark theme tức thì</t>
         </is>
       </c>
     </row>
@@ -970,7 +970,7 @@
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>Hi?n th? d?ng danh s?ch scannable, l?u t?y ch?n hi?n th? v?o localStorage</t>
+          <t>Hiển thị dạng danh sách scannable, lưu tùy chọn hiển thị vào localStorage</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="G19" s="12" t="inlineStr">
         <is>
-          <t>M?c ??nh hi?n th? d?ng l??i responsive (minmax 280px, 1fr)</t>
+          <t>Mặc định hiển thị dạng lưới responsive (minmax 280px, 1fr)</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>Ch? ti?u ?? &amp; n?i dung b?t bu?c; D?NG CHUNG GIAO DI?N V?I S?A GHI CH? (/notes/create -&gt; edit.php)</t>
+          <t>Chỉ tiêu đề &amp; nội dung bắt buộc; DÙNG CHUNG GIAO DIỆN VỚI SỬA GHI CHÚ (/notes/create -&gt; edit.php)</t>
         </is>
       </c>
     </row>
@@ -1063,7 +1063,7 @@
       </c>
       <c r="G21" s="12" t="inlineStr">
         <is>
-          <t>D?NG CHUNG GIAO DI?N V?I T?O GHI CH? (/notes/edit/{id} -&gt; edit.php), ??ng b? realtime</t>
+          <t>DÙNG CHUNG GIAO DIỆN VỚI TẠO GHI CHÚ (/notes/edit/{id} -&gt; edit.php), đồng bộ realtime</t>
         </is>
       </c>
     </row>
@@ -1094,7 +1094,7 @@
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>B?t bu?c c? h?p tho?i x?c nh?n x?a (deleteConfirmModal) ??ng Ti?u ch? 13 Rubric</t>
+          <t>Bắt buộc có hộp thoại xác nhận xóa (deleteConfirmModal) đúng Tiêu chí 13 Rubric</t>
         </is>
       </c>
     </row>
@@ -1125,7 +1125,7 @@
       </c>
       <c r="G23" s="12" t="inlineStr">
         <is>
-          <t>T? ??ng l?u n?i dung ng?m sau khi d?ng g? 0.6s, kh?ng c? n?t 'Save' c?ng</t>
+          <t>Tự động lưu nội dung ngầm sau khi dừng gõ 0.6s, không có nút 'Save' cứng</t>
         </is>
       </c>
     </row>
@@ -1156,7 +1156,7 @@
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>H? tr? ??nh k?m 1 ho?c nhi?u ?nh/video, xem tr??c tr?c ti?p tr?n giao di?n</t>
+          <t>Hỗ trợ đính kèm 1 hoặc nhiều ảnh/video, xem trước trực tiếp trên giao diện</t>
         </is>
       </c>
     </row>
@@ -1187,7 +1187,7 @@
       </c>
       <c r="G25" s="12" t="inlineStr">
         <is>
-          <t>H? tr? t?p ??nh k?m ?a ??nh d?ng (.pdf, .docx, .zip), c? n?t t?i v? v? x?a</t>
+          <t>Hỗ trợ tệp đính kèm đa định dạng (.pdf, .docx, .zip), có nút tải về và xóa</t>
         </is>
       </c>
     </row>
@@ -1218,7 +1218,7 @@
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>S?p x?p theo th?i gian; ghi ch? ghim lu?n ??ng ??u theo th? t? th?i ?i?m ghim (pinned_at)</t>
+          <t>Sắp xếp theo thời gian; ghi chú ghim luôn đứng đầu theo thứ tự thời điểm ghim (pinned_at)</t>
         </is>
       </c>
     </row>
@@ -1249,7 +1249,7 @@
       </c>
       <c r="G27" s="12" t="inlineStr">
         <is>
-          <t>Icon tr?c quan ? c? 2 d?ng l??i v? danh s?ch: Ghim (pin), Kh?a (lock), Chia s? (people)</t>
+          <t>Icon trực quan ở cả 2 dạng lưới và danh sách: Ghim (pin), Khóa (lock), Chia sẻ (people)</t>
         </is>
       </c>
     </row>
@@ -1280,7 +1280,7 @@
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>Qu?t c? ti?u ?? v? n?i dung; Live search 300ms debounce, kh?ng c? n?t Search c?ng; ph?m t?t Ctrl+K, /</t>
+          <t>Quét cả tiêu đề và nội dung; Live search 300ms debounce, không có nút Search cứng; phím tắt Ctrl+K, /</t>
         </is>
       </c>
     </row>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="G29" s="12" t="inlineStr">
         <is>
-          <t>Modal qu?n l? nh?n: xem danh s?ch, t?o m?i, ??i t?n nh?n t?i ch? v? x?a nh?n</t>
+          <t>Modal quản lý nhãn: xem danh sách, tạo mới, đổi tên nhãn tại chỗ và xóa nhãn</t>
         </is>
       </c>
     </row>
@@ -1342,7 +1342,7 @@
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>M?t ghi ch? c? th? kh?ng g?n nh?n ho?c g?n m?t/nhi?u nh?n linh ho?t</t>
+          <t>Một ghi chú có thể không gắn nhãn hoặc gắn một/nhiều nhãn linh hoạt</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1373,7 @@
       </c>
       <c r="G31" s="12" t="inlineStr">
         <is>
-          <t>L?c theo nh?n t? sidebar; x?a nh?n kh?ng m?t ghi ch?; ??i t?n nh?n t? c?p nh?t t?c th?</t>
+          <t>Lọc theo nhãn từ sidebar; xóa nhãn không mất ghi chú; đổi tên nhãn tự cập nhật tức thì</t>
         </is>
       </c>
     </row>
@@ -1404,7 +1404,7 @@
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>B?t kh?a m?t kh?u ri?ng t?ng ghi ch? (nh?p 2 l?n); t?t kh?a y?u c?u nh?p m?t kh?u hi?n t?i</t>
+          <t>Bật khóa mật khẩu riêng từng ghi chú (nhập 2 lần); tắt khóa yêu cầu nhập mật khẩu hiện tại</t>
         </is>
       </c>
     </row>
@@ -1435,7 +1435,7 @@
       </c>
       <c r="G33" s="12" t="inlineStr">
         <is>
-          <t>H?i m?t kh?u tr??c khi Xem/S?a/X?a ghi ch? kh?a; h? tr? ??i m?t kh?u (c? + m?i x2)</t>
+          <t>Hỏi mật khẩu trước khi Xem/Sửa/Xóa ghi chú khóa; hỗ trợ đổi mật khẩu (cũ + mới x2)</t>
         </is>
       </c>
     </row>
@@ -1466,7 +1466,7 @@
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>Chia s? qua email; ph?n quy?n Ch? ??c / S?a; m?c ri?ng '???c chia s? v?i t?i' c? th?i gian &amp; ng??i chia s?</t>
+          <t>Chia sẻ qua email; phân quyền Chỉ đọc / Sửa; mục riêng 'Được chia sẻ với tôi' có thời gian &amp; người chia sẻ</t>
         </is>
       </c>
     </row>
@@ -1497,7 +1497,7 @@
       </c>
       <c r="G35" s="12" t="inlineStr">
         <is>
-          <t>M?y ch? WebSocket thu?n PHP chu?n RFC 6455 (server.php); nhi?u ng??i s?a c?ng th?y thay ??i ngay l?p t?c</t>
+          <t>Máy chủ WebSocket thuần PHP chuẩn RFC 6455 (server.php); nhiều người sửa cùng thấy thay đổi ngay lập tức</t>
         </is>
       </c>
     </row>
@@ -1528,7 +1528,7 @@
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>T?m t?t ghi ch? b?ng LLM c? ??ng, gi? ? ch?nh, c? n?t t?o l?i t?m t?t (AiController.php:summarize)</t>
+          <t>Tóm tắt ghi chú bằng LLM cô đọng, giữ ý chính, có nút tạo lại tóm tắt (AiController.php:summarize)</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1559,7 @@
       </c>
       <c r="G37" s="12" t="inlineStr">
         <is>
-          <t>H?i-??p ng? ngh?a RAG tr?n kho ghi ch?, c?u tr? l?i k?m link tham chi?u m? th?ng ghi ch? ngu?n (/ai)</t>
+          <t>Hỏi-đáp ngữ nghĩa RAG trên kho ghi chú, câu trả lời kèm link tham chiếu mở thẳng ghi chú nguồn (/ai)</t>
         </is>
       </c>
     </row>
@@ -1590,7 +1590,7 @@
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>??t ?i?m tuy?t ??i 40/40 theo 10 Usability Heuristics; WCAG AAA t??ng ph?n 7.1:1; empty/loading/error ??y ??</t>
+          <t>Đạt điểm tuyệt đối 40/40 theo 10 Usability Heuristics; WCAG AAA tương phản 7.1:1; empty/loading/error đầy đủ</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1621,7 @@
       </c>
       <c r="G39" s="12" t="inlineStr">
         <is>
-          <t>T??ng th?ch ho?n h?o Smartphone, Tablet, Desktop; touch target &gt;= 44px; kh?ng tr?n vi?n</t>
+          <t>Tương thích hoàn hảo Smartphone, Tablet, Desktop; touch target &gt;= 44px; không tràn viền</t>
         </is>
       </c>
     </row>
@@ -1652,7 +1652,7 @@
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>PWA Service Worker + IndexedDB xem v? t?m ki?m ghi ch? khi m?t m?ng; t? ??ng ??ng b? khi c? m?ng</t>
+          <t>PWA Service Worker + IndexedDB xem và tìm kiếm ghi chú khi mất mạng; tự động đồng bộ khi có mạng</t>
         </is>
       </c>
     </row>
@@ -1683,14 +1683,14 @@
       </c>
       <c r="G41" s="12" t="inlineStr">
         <is>
-          <t>Docker Compose (docker-compose up -d --build) t? ??ng n?p database v? c?u h?nh s?n s?ng ch?m b?i</t>
+          <t>Docker Compose (docker-compose up -d --build) tự động nạp database và cấu hình sẵn sàng chấm bài</t>
         </is>
       </c>
     </row>
     <row r="42" ht="28" customHeight="1">
       <c r="A42" s="16" t="inlineStr">
         <is>
-          <t>T?NG C?NG ?I?M T? ??NH GI? (32 TI?U CH?):</t>
+          <t>TỔNG CỘNG ĐIỂM TỰ ĐÁNH GIÁ (32 TIÊU CHÍ):</t>
         </is>
       </c>
       <c r="B42" s="17" t="n"/>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="E42" s="18" t="inlineStr">
         <is>
-          <t>100% Ho?n Th?nh</t>
+          <t>100% Hoàn Thành</t>
         </is>
       </c>
       <c r="F42" s="19">
@@ -1710,7 +1710,7 @@
       </c>
       <c r="G42" s="20" t="inlineStr">
         <is>
-          <t>T?t c? 32/32 ti?u ch? ??u ?? ???c c?i ??t v? ki?m th? nghi?m ng?t</t>
+          <t>Tất cả 32/32 tiêu chí đều đã được cài đặt và kiểm thử nghiêm ngặt</t>
         </is>
       </c>
     </row>

</xml_diff>